<commit_message>
feat(v2): V2 PRO — demandes, calcul, visualisation + fix gitignore UTF-8
Nouveaux modules V2 PRO :
- blueprints/pro/demandes.py : gestion des demandes de reception
- services/calculation_service.py : logique calcul conformite
- services/visualization_service.py : rendu resultats
- Templates pro : carte, demandes, simulation, projet_hub, rapport,
  reception_mdc, top_reception, historique_receptions
- Templates admin : projet_visualisation
- Pages : intro.html, landing.html

Mises a jour :
- models.py, __init__.py, api.py, pages.py, admin.py, projets.py
- excel_service, pdf_service, r2_service
- 4 modeles assainissement (P1-P4) mis a jour
- Scripts : migrate_v3-v6, gen_generale, reset_admin_password
- Donnees clients : modeles Excel ajoutes
- Docs : RECEPTA_UI_UX_DOCUMENTATION.md
- Maquettes HTML (html/)

Fix : .gitignore reecrit en UTF-8 — .claude/ desormais correctement ignore

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/modeles_recepta/P2_Urbain_Trottoirs_1.5km.xlsx
+++ b/data/modeles_recepta/P2_Urbain_Trottoirs_1.5km.xlsx
@@ -1,35 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Cote_Gauche" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Cote_Droit" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="LEGENDE" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="PK_Coordonnees" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="OFFSETS_TRANSVERSAUX" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cote_Gauche" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cote_Droit" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IMPREVUS" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PROFIL_LONG" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SECTIONS" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LEGENDE" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'PK_Coordonnees'!$A$3:$F$65</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
-    <numFmt numFmtId="164" formatCode="#,##0.000"/>
-    <numFmt numFmtId="165" formatCode="0.000"/>
-    <numFmt numFmtId="166" formatCode="0.0000"/>
-    <numFmt numFmtId="167" formatCode="0.0"/>
-    <numFmt numFmtId="168" formatCode="+0.000;-0.000;0.000"/>
-  </numFmts>
-  <fonts count="21">
+  <numFmts count="0"/>
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -52,6 +45,24 @@
       <sz val="9"/>
     </font>
     <font>
+      <color rgb="0092400E"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <color rgb="009CA3AF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="006B7280"/>
+      <sz val="7"/>
+    </font>
+    <font>
       <b val="1"/>
       <color rgb="0000FFFF"/>
       <sz val="12"/>
@@ -72,77 +83,8 @@
       <color rgb="00FFFFFF"/>
       <sz val="9"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="00475569"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="0064748B"/>
-      <sz val="8"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="001E3A5F"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="001E293B"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="00B45309"/>
-      <sz val="8"/>
-    </font>
-    <font>
-      <name val="Courier New"/>
-      <b val="1"/>
-      <color rgb="000F4C35"/>
-      <sz val="8"/>
-    </font>
-    <font>
-      <name val="Courier New"/>
-      <color rgb="00475569"/>
-      <sz val="8"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="000F766E"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="000F766E"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="001E3A5F"/>
-      <sz val="8"/>
-    </font>
   </fonts>
-  <fills count="25">
+  <fills count="23">
     <fill>
       <patternFill/>
     </fill>
@@ -211,27 +153,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000D1F38"/>
+        <fgColor rgb="00F59E0B"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8FAFC"/>
+        <fgColor rgb="00FFF8E1"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F1F5F9"/>
+        <fgColor rgb="00DBEAFE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EFF6FF"/>
+        <fgColor rgb="00374151"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
+        <fgColor rgb="004B5563"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0F9FF"/>
       </patternFill>
     </fill>
     <fill>
@@ -241,31 +188,16 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000F4C35"/>
+        <fgColor rgb="00F9FAFB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F0FDF4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E0FFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FEE2E2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DBEAFE"/>
+        <fgColor rgb="000D1F38"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -289,23 +221,51 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="00FCD34D"/>
       </left>
       <right style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="00FCD34D"/>
       </right>
       <top style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="00FCD34D"/>
       </top>
       <bottom style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="00FCD34D"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="0093C5FD"/>
+      </left>
+      <right style="thin">
+        <color rgb="0093C5FD"/>
+      </right>
+      <top style="thin">
+        <color rgb="0093C5FD"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="0093C5FD"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D1D5DB"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D1D5DB"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -343,125 +303,87 @@
     <xf numFmtId="0" fontId="3" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" indent="1"/>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" indent="1"/>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" indent="1"/>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" indent="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" indent="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" indent="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" indent="1"/>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" indent="1"/>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" indent="1"/>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" indent="1"/>
+    <xf numFmtId="0" fontId="1" fillId="18" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" indent="1"/>
+    <xf numFmtId="0" fontId="2" fillId="19" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" indent="1"/>
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="166" fontId="13" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="167" fontId="13" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="18" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="18" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="18" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="14" fillId="18" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="14" fillId="18" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="20" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="22" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="18" fillId="22" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="23" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="14" fillId="23" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="24" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="14" fillId="24" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -537,6 +459,36 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="9334500" cy="3429000"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6833,6 +6785,1233 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:Y4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
+    <col width="13" customWidth="1" min="20" max="20"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="22" max="22"/>
+    <col width="13" customWidth="1" min="23" max="23"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="25" max="25"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="40" customHeight="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="B1" s="13" t="inlineStr">
+        <is>
+          <t>AXE_BB</t>
+        </is>
+      </c>
+      <c r="C1" s="13" t="inlineStr">
+        <is>
+          <t>AXE_Travaux</t>
+        </is>
+      </c>
+      <c r="D1" s="13" t="inlineStr">
+        <is>
+          <t>AXE_Fond_Forme</t>
+        </is>
+      </c>
+      <c r="E1" s="13" t="inlineStr">
+        <is>
+          <t>G_BB_Roulement</t>
+        </is>
+      </c>
+      <c r="F1" s="13" t="inlineStr">
+        <is>
+          <t>G_Travaux_Base</t>
+        </is>
+      </c>
+      <c r="G1" s="13" t="inlineStr">
+        <is>
+          <t>G_Fond_Forme</t>
+        </is>
+      </c>
+      <c r="H1" s="13" t="inlineStr">
+        <is>
+          <t>G_Bordure_Finie</t>
+        </is>
+      </c>
+      <c r="I1" s="13" t="inlineStr">
+        <is>
+          <t>G_Bord_Stationnement</t>
+        </is>
+      </c>
+      <c r="J1" s="13" t="inlineStr">
+        <is>
+          <t>G_Trottoir_Fini</t>
+        </is>
+      </c>
+      <c r="K1" s="13" t="inlineStr">
+        <is>
+          <t>G_Tablier_Fini_60x60</t>
+        </is>
+      </c>
+      <c r="L1" s="13" t="inlineStr">
+        <is>
+          <t>G_Radier_Interieur</t>
+        </is>
+      </c>
+      <c r="M1" s="13" t="inlineStr">
+        <is>
+          <t>G_Beton_Proprete</t>
+        </is>
+      </c>
+      <c r="N1" s="13" t="inlineStr">
+        <is>
+          <t>G_Fond_Fouille</t>
+        </is>
+      </c>
+      <c r="O1" s="13" t="inlineStr">
+        <is>
+          <t>G_Bord_Propriete</t>
+        </is>
+      </c>
+      <c r="P1" s="13" t="inlineStr">
+        <is>
+          <t>D_BB_Roulement</t>
+        </is>
+      </c>
+      <c r="Q1" s="13" t="inlineStr">
+        <is>
+          <t>D_Travaux_Base</t>
+        </is>
+      </c>
+      <c r="R1" s="13" t="inlineStr">
+        <is>
+          <t>D_Fond_Forme</t>
+        </is>
+      </c>
+      <c r="S1" s="13" t="inlineStr">
+        <is>
+          <t>D_Bordure_Finie</t>
+        </is>
+      </c>
+      <c r="T1" s="13" t="inlineStr">
+        <is>
+          <t>D_Trottoir_Fini</t>
+        </is>
+      </c>
+      <c r="U1" s="13" t="inlineStr">
+        <is>
+          <t>D_Tablier_Fini_40x40</t>
+        </is>
+      </c>
+      <c r="V1" s="13" t="inlineStr">
+        <is>
+          <t>D_Radier_Interieur</t>
+        </is>
+      </c>
+      <c r="W1" s="13" t="inlineStr">
+        <is>
+          <t>D_Beton_Proprete</t>
+        </is>
+      </c>
+      <c r="X1" s="13" t="inlineStr">
+        <is>
+          <t>D_Fond_Fouille</t>
+        </is>
+      </c>
+      <c r="Y1" s="13" t="inlineStr">
+        <is>
+          <t>D_Bord_Propriete</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="14" customHeight="1">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>0+012</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="n">
+        <v>98.29600000000001</v>
+      </c>
+      <c r="C2" s="15" t="n">
+        <v>98.236</v>
+      </c>
+      <c r="D2" s="15" t="n">
+        <v>98.036</v>
+      </c>
+      <c r="E2" s="15" t="n">
+        <v>98.226</v>
+      </c>
+      <c r="F2" s="15" t="n">
+        <v>98.166</v>
+      </c>
+      <c r="G2" s="15" t="n">
+        <v>97.96599999999999</v>
+      </c>
+      <c r="H2" s="15" t="n">
+        <v>98.206</v>
+      </c>
+      <c r="I2" s="15" t="n">
+        <v>98.18600000000001</v>
+      </c>
+      <c r="J2" s="15" t="n">
+        <v>98.256</v>
+      </c>
+      <c r="K2" s="15" t="n">
+        <v>98.226</v>
+      </c>
+      <c r="L2" s="15" t="n">
+        <v>97.526</v>
+      </c>
+      <c r="M2" s="15" t="n">
+        <v>97.426</v>
+      </c>
+      <c r="N2" s="15" t="n">
+        <v>97.226</v>
+      </c>
+      <c r="O2" s="15" t="n">
+        <v>98.426</v>
+      </c>
+      <c r="P2" s="15" t="n">
+        <v>98.191</v>
+      </c>
+      <c r="Q2" s="15" t="n">
+        <v>98.131</v>
+      </c>
+      <c r="R2" s="15" t="n">
+        <v>97.931</v>
+      </c>
+      <c r="S2" s="15" t="n">
+        <v>98.17100000000001</v>
+      </c>
+      <c r="T2" s="15" t="n">
+        <v>98.251</v>
+      </c>
+      <c r="U2" s="15" t="n">
+        <v>98.191</v>
+      </c>
+      <c r="V2" s="15" t="n">
+        <v>97.691</v>
+      </c>
+      <c r="W2" s="15" t="n">
+        <v>97.59099999999999</v>
+      </c>
+      <c r="X2" s="15" t="n">
+        <v>97.39100000000001</v>
+      </c>
+      <c r="Y2" s="15" t="n">
+        <v>98.39100000000001</v>
+      </c>
+    </row>
+    <row r="3" ht="14" customHeight="1">
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>0+040</t>
+        </is>
+      </c>
+      <c r="B3" s="15" t="n">
+        <v>98.52</v>
+      </c>
+      <c r="C3" s="15" t="n">
+        <v>98.45999999999999</v>
+      </c>
+      <c r="D3" s="15" t="n">
+        <v>98.26000000000001</v>
+      </c>
+      <c r="E3" s="15" t="n">
+        <v>98.45</v>
+      </c>
+      <c r="F3" s="15" t="n">
+        <v>98.39</v>
+      </c>
+      <c r="G3" s="15" t="n">
+        <v>98.19</v>
+      </c>
+      <c r="H3" s="15" t="n">
+        <v>98.43000000000001</v>
+      </c>
+      <c r="I3" s="15" t="n">
+        <v>98.41</v>
+      </c>
+      <c r="J3" s="15" t="n">
+        <v>98.48</v>
+      </c>
+      <c r="K3" s="15" t="n">
+        <v>98.45</v>
+      </c>
+      <c r="L3" s="15" t="n">
+        <v>97.75</v>
+      </c>
+      <c r="M3" s="15" t="n">
+        <v>97.65000000000001</v>
+      </c>
+      <c r="N3" s="15" t="n">
+        <v>97.45</v>
+      </c>
+      <c r="O3" s="15" t="n">
+        <v>98.65000000000001</v>
+      </c>
+      <c r="P3" s="15" t="n">
+        <v>98.41500000000001</v>
+      </c>
+      <c r="Q3" s="15" t="n">
+        <v>98.355</v>
+      </c>
+      <c r="R3" s="15" t="n">
+        <v>98.155</v>
+      </c>
+      <c r="S3" s="15" t="n">
+        <v>98.395</v>
+      </c>
+      <c r="T3" s="15" t="n">
+        <v>98.47499999999999</v>
+      </c>
+      <c r="U3" s="15" t="n">
+        <v>98.41500000000001</v>
+      </c>
+      <c r="V3" s="15" t="n">
+        <v>97.91500000000001</v>
+      </c>
+      <c r="W3" s="15" t="n">
+        <v>97.815</v>
+      </c>
+      <c r="X3" s="15" t="n">
+        <v>97.61499999999999</v>
+      </c>
+      <c r="Y3" s="15" t="n">
+        <v>98.61499999999999</v>
+      </c>
+    </row>
+    <row r="4" ht="14" customHeight="1">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>0+068</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="n">
+        <v>98.744</v>
+      </c>
+      <c r="C4" s="15" t="n">
+        <v>98.684</v>
+      </c>
+      <c r="D4" s="15" t="n">
+        <v>98.48399999999999</v>
+      </c>
+      <c r="E4" s="15" t="n">
+        <v>98.67400000000001</v>
+      </c>
+      <c r="F4" s="15" t="n">
+        <v>98.614</v>
+      </c>
+      <c r="G4" s="15" t="n">
+        <v>98.414</v>
+      </c>
+      <c r="H4" s="15" t="n">
+        <v>98.654</v>
+      </c>
+      <c r="I4" s="15" t="n">
+        <v>98.634</v>
+      </c>
+      <c r="J4" s="15" t="n">
+        <v>98.70399999999999</v>
+      </c>
+      <c r="K4" s="15" t="n">
+        <v>98.67400000000001</v>
+      </c>
+      <c r="L4" s="15" t="n">
+        <v>97.974</v>
+      </c>
+      <c r="M4" s="15" t="n">
+        <v>97.874</v>
+      </c>
+      <c r="N4" s="15" t="n">
+        <v>97.67400000000001</v>
+      </c>
+      <c r="O4" s="15" t="n">
+        <v>98.874</v>
+      </c>
+      <c r="P4" s="15" t="n">
+        <v>98.639</v>
+      </c>
+      <c r="Q4" s="15" t="n">
+        <v>98.57899999999999</v>
+      </c>
+      <c r="R4" s="15" t="n">
+        <v>98.379</v>
+      </c>
+      <c r="S4" s="15" t="n">
+        <v>98.619</v>
+      </c>
+      <c r="T4" s="15" t="n">
+        <v>98.699</v>
+      </c>
+      <c r="U4" s="15" t="n">
+        <v>98.639</v>
+      </c>
+      <c r="V4" s="15" t="n">
+        <v>98.139</v>
+      </c>
+      <c r="W4" s="15" t="n">
+        <v>98.039</v>
+      </c>
+      <c r="X4" s="15" t="n">
+        <v>97.839</v>
+      </c>
+      <c r="Y4" s="15" t="n">
+        <v>98.839</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B62"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="B1" s="16" t="inlineStr">
+        <is>
+          <t>Z_axe (m NGF)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="14" customHeight="1">
+      <c r="A2" s="17" t="inlineStr">
+        <is>
+          <t>0+000</t>
+        </is>
+      </c>
+      <c r="B2" s="18" t="n">
+        <v>98.2</v>
+      </c>
+    </row>
+    <row r="3" ht="14" customHeight="1">
+      <c r="A3" s="19" t="inlineStr">
+        <is>
+          <t>0+025</t>
+        </is>
+      </c>
+      <c r="B3" s="20" t="n">
+        <v>98.40000000000001</v>
+      </c>
+    </row>
+    <row r="4" ht="14" customHeight="1">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>0+050</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="n">
+        <v>98.59999999999999</v>
+      </c>
+    </row>
+    <row r="5" ht="14" customHeight="1">
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>0+075</t>
+        </is>
+      </c>
+      <c r="B5" s="20" t="n">
+        <v>98.8</v>
+      </c>
+    </row>
+    <row r="6" ht="14" customHeight="1">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>0+100</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="7" ht="14" customHeight="1">
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>0+125</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="n">
+        <v>99.2</v>
+      </c>
+    </row>
+    <row r="8" ht="14" customHeight="1">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>0+150</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="n">
+        <v>99.40000000000001</v>
+      </c>
+    </row>
+    <row r="9" ht="14" customHeight="1">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>0+175</t>
+        </is>
+      </c>
+      <c r="B9" s="20" t="n">
+        <v>99.59999999999999</v>
+      </c>
+    </row>
+    <row r="10" ht="14" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>0+200</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="n">
+        <v>99.8</v>
+      </c>
+    </row>
+    <row r="11" ht="14" customHeight="1">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>0+225</t>
+        </is>
+      </c>
+      <c r="B11" s="20" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="12" ht="14" customHeight="1">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>0+250</t>
+        </is>
+      </c>
+      <c r="B12" s="18" t="n">
+        <v>100.2</v>
+      </c>
+    </row>
+    <row r="13" ht="14" customHeight="1">
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>0+275</t>
+        </is>
+      </c>
+      <c r="B13" s="20" t="n">
+        <v>100.4</v>
+      </c>
+    </row>
+    <row r="14" ht="14" customHeight="1">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>0+300</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="n">
+        <v>100.6</v>
+      </c>
+    </row>
+    <row r="15" ht="14" customHeight="1">
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>0+325</t>
+        </is>
+      </c>
+      <c r="B15" s="20" t="n">
+        <v>100.8</v>
+      </c>
+    </row>
+    <row r="16" ht="14" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>0+350</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="n">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="17" ht="14" customHeight="1">
+      <c r="A17" s="19" t="inlineStr">
+        <is>
+          <t>0+375</t>
+        </is>
+      </c>
+      <c r="B17" s="20" t="n">
+        <v>101.2</v>
+      </c>
+    </row>
+    <row r="18" ht="14" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>0+400</t>
+        </is>
+      </c>
+      <c r="B18" s="18" t="n">
+        <v>101.4</v>
+      </c>
+    </row>
+    <row r="19" ht="14" customHeight="1">
+      <c r="A19" s="19" t="inlineStr">
+        <is>
+          <t>0+425</t>
+        </is>
+      </c>
+      <c r="B19" s="20" t="n">
+        <v>101.6</v>
+      </c>
+    </row>
+    <row r="20" ht="14" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>0+450</t>
+        </is>
+      </c>
+      <c r="B20" s="18" t="n">
+        <v>101.8</v>
+      </c>
+    </row>
+    <row r="21" ht="14" customHeight="1">
+      <c r="A21" s="19" t="inlineStr">
+        <is>
+          <t>0+475</t>
+        </is>
+      </c>
+      <c r="B21" s="20" t="n">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="22" ht="14" customHeight="1">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>0+500</t>
+        </is>
+      </c>
+      <c r="B22" s="18" t="n">
+        <v>102.2</v>
+      </c>
+    </row>
+    <row r="23" ht="14" customHeight="1">
+      <c r="A23" s="19" t="inlineStr">
+        <is>
+          <t>0+525</t>
+        </is>
+      </c>
+      <c r="B23" s="20" t="n">
+        <v>102.4</v>
+      </c>
+    </row>
+    <row r="24" ht="14" customHeight="1">
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t>0+550</t>
+        </is>
+      </c>
+      <c r="B24" s="18" t="n">
+        <v>102.6</v>
+      </c>
+    </row>
+    <row r="25" ht="14" customHeight="1">
+      <c r="A25" s="19" t="inlineStr">
+        <is>
+          <t>0+575</t>
+        </is>
+      </c>
+      <c r="B25" s="20" t="n">
+        <v>102.8</v>
+      </c>
+    </row>
+    <row r="26" ht="14" customHeight="1">
+      <c r="A26" s="17" t="inlineStr">
+        <is>
+          <t>0+600</t>
+        </is>
+      </c>
+      <c r="B26" s="18" t="n">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="27" ht="14" customHeight="1">
+      <c r="A27" s="19" t="inlineStr">
+        <is>
+          <t>0+625</t>
+        </is>
+      </c>
+      <c r="B27" s="20" t="n">
+        <v>103.2</v>
+      </c>
+    </row>
+    <row r="28" ht="14" customHeight="1">
+      <c r="A28" s="17" t="inlineStr">
+        <is>
+          <t>0+650</t>
+        </is>
+      </c>
+      <c r="B28" s="18" t="n">
+        <v>103.4</v>
+      </c>
+    </row>
+    <row r="29" ht="14" customHeight="1">
+      <c r="A29" s="19" t="inlineStr">
+        <is>
+          <t>0+675</t>
+        </is>
+      </c>
+      <c r="B29" s="20" t="n">
+        <v>103.6</v>
+      </c>
+    </row>
+    <row r="30" ht="14" customHeight="1">
+      <c r="A30" s="17" t="inlineStr">
+        <is>
+          <t>0+700</t>
+        </is>
+      </c>
+      <c r="B30" s="18" t="n">
+        <v>103.8</v>
+      </c>
+    </row>
+    <row r="31" ht="14" customHeight="1">
+      <c r="A31" s="19" t="inlineStr">
+        <is>
+          <t>0+725</t>
+        </is>
+      </c>
+      <c r="B31" s="20" t="n">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="32" ht="14" customHeight="1">
+      <c r="A32" s="17" t="inlineStr">
+        <is>
+          <t>0+750</t>
+        </is>
+      </c>
+      <c r="B32" s="18" t="n">
+        <v>104.2</v>
+      </c>
+    </row>
+    <row r="33" ht="14" customHeight="1">
+      <c r="A33" s="19" t="inlineStr">
+        <is>
+          <t>0+775</t>
+        </is>
+      </c>
+      <c r="B33" s="20" t="n">
+        <v>104.4</v>
+      </c>
+    </row>
+    <row r="34" ht="14" customHeight="1">
+      <c r="A34" s="17" t="inlineStr">
+        <is>
+          <t>0+800</t>
+        </is>
+      </c>
+      <c r="B34" s="18" t="n">
+        <v>104.6</v>
+      </c>
+    </row>
+    <row r="35" ht="14" customHeight="1">
+      <c r="A35" s="19" t="inlineStr">
+        <is>
+          <t>0+825</t>
+        </is>
+      </c>
+      <c r="B35" s="20" t="n">
+        <v>104.8</v>
+      </c>
+    </row>
+    <row r="36" ht="14" customHeight="1">
+      <c r="A36" s="17" t="inlineStr">
+        <is>
+          <t>0+850</t>
+        </is>
+      </c>
+      <c r="B36" s="18" t="n">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="37" ht="14" customHeight="1">
+      <c r="A37" s="19" t="inlineStr">
+        <is>
+          <t>0+875</t>
+        </is>
+      </c>
+      <c r="B37" s="20" t="n">
+        <v>105.2</v>
+      </c>
+    </row>
+    <row r="38" ht="14" customHeight="1">
+      <c r="A38" s="17" t="inlineStr">
+        <is>
+          <t>0+900</t>
+        </is>
+      </c>
+      <c r="B38" s="18" t="n">
+        <v>105.4</v>
+      </c>
+    </row>
+    <row r="39" ht="14" customHeight="1">
+      <c r="A39" s="19" t="inlineStr">
+        <is>
+          <t>0+925</t>
+        </is>
+      </c>
+      <c r="B39" s="20" t="n">
+        <v>105.6</v>
+      </c>
+    </row>
+    <row r="40" ht="14" customHeight="1">
+      <c r="A40" s="17" t="inlineStr">
+        <is>
+          <t>0+950</t>
+        </is>
+      </c>
+      <c r="B40" s="18" t="n">
+        <v>105.8</v>
+      </c>
+    </row>
+    <row r="41" ht="14" customHeight="1">
+      <c r="A41" s="19" t="inlineStr">
+        <is>
+          <t>0+975</t>
+        </is>
+      </c>
+      <c r="B41" s="20" t="n">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="42" ht="14" customHeight="1">
+      <c r="A42" s="17" t="inlineStr">
+        <is>
+          <t>1+000</t>
+        </is>
+      </c>
+      <c r="B42" s="18" t="n">
+        <v>106.2</v>
+      </c>
+    </row>
+    <row r="43" ht="14" customHeight="1">
+      <c r="A43" s="19" t="inlineStr">
+        <is>
+          <t>1+025</t>
+        </is>
+      </c>
+      <c r="B43" s="20" t="n">
+        <v>106.4</v>
+      </c>
+    </row>
+    <row r="44" ht="14" customHeight="1">
+      <c r="A44" s="17" t="inlineStr">
+        <is>
+          <t>1+050</t>
+        </is>
+      </c>
+      <c r="B44" s="18" t="n">
+        <v>106.6</v>
+      </c>
+    </row>
+    <row r="45" ht="14" customHeight="1">
+      <c r="A45" s="19" t="inlineStr">
+        <is>
+          <t>1+075</t>
+        </is>
+      </c>
+      <c r="B45" s="20" t="n">
+        <v>106.8</v>
+      </c>
+    </row>
+    <row r="46" ht="14" customHeight="1">
+      <c r="A46" s="17" t="inlineStr">
+        <is>
+          <t>1+100</t>
+        </is>
+      </c>
+      <c r="B46" s="18" t="n">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="47" ht="14" customHeight="1">
+      <c r="A47" s="19" t="inlineStr">
+        <is>
+          <t>1+125</t>
+        </is>
+      </c>
+      <c r="B47" s="20" t="n">
+        <v>107.2</v>
+      </c>
+    </row>
+    <row r="48" ht="14" customHeight="1">
+      <c r="A48" s="17" t="inlineStr">
+        <is>
+          <t>1+150</t>
+        </is>
+      </c>
+      <c r="B48" s="18" t="n">
+        <v>107.4</v>
+      </c>
+    </row>
+    <row r="49" ht="14" customHeight="1">
+      <c r="A49" s="19" t="inlineStr">
+        <is>
+          <t>1+175</t>
+        </is>
+      </c>
+      <c r="B49" s="20" t="n">
+        <v>107.6</v>
+      </c>
+    </row>
+    <row r="50" ht="14" customHeight="1">
+      <c r="A50" s="17" t="inlineStr">
+        <is>
+          <t>1+200</t>
+        </is>
+      </c>
+      <c r="B50" s="18" t="n">
+        <v>107.8</v>
+      </c>
+    </row>
+    <row r="51" ht="14" customHeight="1">
+      <c r="A51" s="19" t="inlineStr">
+        <is>
+          <t>1+225</t>
+        </is>
+      </c>
+      <c r="B51" s="20" t="n">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="52" ht="14" customHeight="1">
+      <c r="A52" s="17" t="inlineStr">
+        <is>
+          <t>1+250</t>
+        </is>
+      </c>
+      <c r="B52" s="18" t="n">
+        <v>108.2</v>
+      </c>
+    </row>
+    <row r="53" ht="14" customHeight="1">
+      <c r="A53" s="19" t="inlineStr">
+        <is>
+          <t>1+275</t>
+        </is>
+      </c>
+      <c r="B53" s="20" t="n">
+        <v>108.4</v>
+      </c>
+    </row>
+    <row r="54" ht="14" customHeight="1">
+      <c r="A54" s="17" t="inlineStr">
+        <is>
+          <t>1+300</t>
+        </is>
+      </c>
+      <c r="B54" s="18" t="n">
+        <v>108.6</v>
+      </c>
+    </row>
+    <row r="55" ht="14" customHeight="1">
+      <c r="A55" s="19" t="inlineStr">
+        <is>
+          <t>1+325</t>
+        </is>
+      </c>
+      <c r="B55" s="20" t="n">
+        <v>108.8</v>
+      </c>
+    </row>
+    <row r="56" ht="14" customHeight="1">
+      <c r="A56" s="17" t="inlineStr">
+        <is>
+          <t>1+350</t>
+        </is>
+      </c>
+      <c r="B56" s="18" t="n">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="57" ht="14" customHeight="1">
+      <c r="A57" s="19" t="inlineStr">
+        <is>
+          <t>1+375</t>
+        </is>
+      </c>
+      <c r="B57" s="20" t="n">
+        <v>109.2</v>
+      </c>
+    </row>
+    <row r="58" ht="14" customHeight="1">
+      <c r="A58" s="17" t="inlineStr">
+        <is>
+          <t>1+400</t>
+        </is>
+      </c>
+      <c r="B58" s="18" t="n">
+        <v>109.4</v>
+      </c>
+    </row>
+    <row r="59" ht="14" customHeight="1">
+      <c r="A59" s="19" t="inlineStr">
+        <is>
+          <t>1+425</t>
+        </is>
+      </c>
+      <c r="B59" s="20" t="n">
+        <v>109.6</v>
+      </c>
+    </row>
+    <row r="60" ht="14" customHeight="1">
+      <c r="A60" s="17" t="inlineStr">
+        <is>
+          <t>1+450</t>
+        </is>
+      </c>
+      <c r="B60" s="18" t="n">
+        <v>109.8</v>
+      </c>
+    </row>
+    <row r="61" ht="14" customHeight="1">
+      <c r="A61" s="19" t="inlineStr">
+        <is>
+          <t>1+475</t>
+        </is>
+      </c>
+      <c r="B61" s="20" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="62" ht="14" customHeight="1">
+      <c r="A62" s="17" t="inlineStr">
+        <is>
+          <t>1+500</t>
+        </is>
+      </c>
+      <c r="B62" s="18" t="n">
+        <v>110.2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="18" customHeight="1">
+      <c r="A1" s="21" t="inlineStr">
+        <is>
+          <t>SECTIONS — Paramètres variables par tronçon  |  Ajouter une ligne si épaisseurs / dévers / distances changent</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="22" t="inlineStr">
+        <is>
+          <t>Num</t>
+        </is>
+      </c>
+      <c r="B2" s="22" t="inlineStr">
+        <is>
+          <t>Nom_Section</t>
+        </is>
+      </c>
+      <c r="C2" s="22" t="inlineStr">
+        <is>
+          <t>PK_debut</t>
+        </is>
+      </c>
+      <c r="D2" s="22" t="inlineStr">
+        <is>
+          <t>PK_fin</t>
+        </is>
+      </c>
+      <c r="E2" s="22" t="inlineStr">
+        <is>
+          <t>e_BB_m</t>
+        </is>
+      </c>
+      <c r="F2" s="22" t="inlineStr">
+        <is>
+          <t>e_GB4_m</t>
+        </is>
+      </c>
+      <c r="G2" s="22" t="inlineStr">
+        <is>
+          <t>e_GNT_m</t>
+        </is>
+      </c>
+      <c r="H2" s="22" t="inlineStr">
+        <is>
+          <t>e_FF_m</t>
+        </is>
+      </c>
+      <c r="I2" s="22" t="inlineStr">
+        <is>
+          <t>Devers_G_pct</t>
+        </is>
+      </c>
+      <c r="J2" s="22" t="inlineStr">
+        <is>
+          <t>Devers_D_pct</t>
+        </is>
+      </c>
+      <c r="K2" s="22" t="inlineStr">
+        <is>
+          <t>Dist_G_m</t>
+        </is>
+      </c>
+      <c r="L2" s="22" t="inlineStr">
+        <is>
+          <t>Dist_D_m</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1">
+      <c r="A3" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="23" t="inlineStr">
+        <is>
+          <t>Section principale</t>
+        </is>
+      </c>
+      <c r="C3" s="24" t="inlineStr">
+        <is>
+          <t>0+000</t>
+        </is>
+      </c>
+      <c r="D3" s="24" t="inlineStr">
+        <is>
+          <t>1+500</t>
+        </is>
+      </c>
+      <c r="E3" s="24" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="F3" s="24" t="n"/>
+      <c r="G3" s="24" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="H3" s="24" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="I3" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="J3" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="K3" s="24" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="L3" s="24" t="n">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="4" ht="14" customHeight="1">
+      <c r="A4" s="25" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="26" t="inlineStr"/>
+      <c r="C4" s="26" t="inlineStr"/>
+      <c r="D4" s="26" t="inlineStr"/>
+      <c r="E4" s="26" t="inlineStr"/>
+      <c r="F4" s="26" t="inlineStr"/>
+      <c r="G4" s="26" t="inlineStr"/>
+      <c r="H4" s="26" t="inlineStr"/>
+      <c r="I4" s="26" t="inlineStr"/>
+      <c r="J4" s="26" t="inlineStr"/>
+      <c r="K4" s="26" t="inlineStr"/>
+      <c r="L4" s="26" t="inlineStr"/>
+    </row>
+    <row r="5" ht="14" customHeight="1">
+      <c r="A5" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="26" t="inlineStr"/>
+      <c r="C5" s="26" t="inlineStr"/>
+      <c r="D5" s="26" t="inlineStr"/>
+      <c r="E5" s="26" t="inlineStr"/>
+      <c r="F5" s="26" t="inlineStr"/>
+      <c r="G5" s="26" t="inlineStr"/>
+      <c r="H5" s="26" t="inlineStr"/>
+      <c r="I5" s="26" t="inlineStr"/>
+      <c r="J5" s="26" t="inlineStr"/>
+      <c r="K5" s="26" t="inlineStr"/>
+      <c r="L5" s="26" t="inlineStr"/>
+    </row>
+    <row r="6" ht="14" customHeight="1">
+      <c r="A6" s="27" t="inlineStr">
+        <is>
+          <t>Légende : e_BB/GB4/GNT/FF en mètres  |  Devers_G/D en %  |  Dist_G/D = distance axe→bord en m  |  e_GB4 vide = couche absente</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A6:L6"/>
+    <mergeCell ref="A1:L1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="B25:B78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -6864,359 +8043,359 @@
     <row r="23" ht="17" customHeight="1"/>
     <row r="24" ht="17" customHeight="1"/>
     <row r="25" ht="17" customHeight="1">
-      <c r="B25" s="13" t="inlineStr">
+      <c r="B25" s="28" t="inlineStr">
         <is>
           <t>SPECIFICATIONS DU PROJET</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
-      <c r="B26" s="14" t="inlineStr">
+      <c r="B26" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">  Titre:          Route Urbaine trottoirs + stationnement</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1">
-      <c r="B27" s="14" t="inlineStr">
+      <c r="B27" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">  Devers:         G:2.0% | D:3.0%</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
-      <c r="B28" s="14" t="inlineStr">
+      <c r="B28" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">  Largeurs:       G: chaussee 3.5m + stat 2.0m + trottoir 1.5m | D: chaussee 3.5m + trottoir 2.0m</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
-      <c r="B29" s="14" t="inlineStr">
+      <c r="B29" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">  Couches:        BB 6cm / Travaux 20cm / Fond de Forme 25cm</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
-      <c r="B30" s="14" t="inlineStr">
+      <c r="B30" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">  Pente long.:    0.8%</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
-      <c r="B31" s="14" t="inlineStr">
+      <c r="B31" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">  Cote axe Z0:    98.200 m NGF</t>
         </is>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
-      <c r="B32" s="14" t="inlineStr">
+      <c r="B32" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">  PK debut/fin:   0+000 / 1+500</t>
         </is>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1">
-      <c r="B33" s="14" t="inlineStr">
+      <c r="B33" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">  Pas PK:         25 m</t>
         </is>
       </c>
     </row>
     <row r="35" ht="11" customHeight="1">
-      <c r="B35" s="15" t="inlineStr"/>
+      <c r="B35" s="30" t="inlineStr"/>
     </row>
     <row r="36" ht="15" customHeight="1">
-      <c r="B36" s="16" t="inlineStr">
+      <c r="B36" s="31" t="inlineStr">
         <is>
           <t>ASSAINISSEMENT GAUCHE — 60x60 (H=0.60m)</t>
         </is>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
-      <c r="B37" s="17" t="inlineStr">
+      <c r="B37" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve">  Caniveau ferme 60x60 — H int=0.60m / dalle=10cm / radier=10cm / BP=20cm</t>
         </is>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
-      <c r="B38" s="18" t="inlineStr">
+      <c r="B38" s="33" t="inlineStr">
         <is>
           <t>ASSAINISSEMENT DROIT  — 40x40 (H=0.40m)</t>
         </is>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
-      <c r="B39" s="19" t="inlineStr">
+      <c r="B39" s="34" t="inlineStr">
         <is>
           <t xml:space="preserve">  Caniveau ferme 40x40 — H int=0.40m / dalle=10cm / radier=10cm / BP=20cm</t>
         </is>
       </c>
     </row>
     <row r="40" ht="11" customHeight="1">
-      <c r="B40" s="15" t="inlineStr"/>
+      <c r="B40" s="30" t="inlineStr"/>
     </row>
     <row r="41" ht="15" customHeight="1">
-      <c r="B41" s="20" t="inlineStr">
+      <c r="B41" s="35" t="inlineStr">
         <is>
           <t>STRATIGRAPHIE ASSAINISSEMENT (de bas en haut) :</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
-      <c r="B42" s="21" t="inlineStr">
+      <c r="B42" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve">  Fond de Fouille                         (cote la plus basse)</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
-      <c r="B43" s="21" t="inlineStr">
+      <c r="B43" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve">  + 20 cm  → Beton de Proprete (BP)       dessus de la couche de 20cm</t>
         </is>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1">
-      <c r="B44" s="21" t="inlineStr">
+      <c r="B44" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve">  + 10 cm  → Radier Interieur             interieur fond du caniveau</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
-      <c r="B45" s="21" t="inlineStr">
+      <c r="B45" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve">  + H canal (100 / 80 / 60 / 50 cm...)   hauteur utile interieure</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1">
-      <c r="B46" s="21" t="inlineStr">
+      <c r="B46" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve">  + e dalle                               Tablier Fini = bord chaussee</t>
         </is>
       </c>
     </row>
     <row r="47" ht="11" customHeight="1">
-      <c r="B47" s="15" t="inlineStr"/>
+      <c r="B47" s="30" t="inlineStr"/>
     </row>
     <row r="48" ht="15" customHeight="1">
-      <c r="B48" s="22" t="inlineStr">
+      <c r="B48" s="37" t="inlineStr">
         <is>
           <t>COLONNES COTE_GAUCHE</t>
         </is>
       </c>
     </row>
     <row r="49" ht="14" customHeight="1">
-      <c r="B49" s="23" t="inlineStr">
+      <c r="B49" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  PK</t>
         </is>
       </c>
     </row>
     <row r="50" ht="14" customHeight="1">
-      <c r="B50" s="23" t="inlineStr">
+      <c r="B50" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  AXE_BB</t>
         </is>
       </c>
     </row>
     <row r="51" ht="14" customHeight="1">
-      <c r="B51" s="23" t="inlineStr">
+      <c r="B51" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  AXE_Travaux</t>
         </is>
       </c>
     </row>
     <row r="52" ht="14" customHeight="1">
-      <c r="B52" s="23" t="inlineStr">
+      <c r="B52" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  AXE_Fond_Forme</t>
         </is>
       </c>
     </row>
     <row r="53" ht="14" customHeight="1">
-      <c r="B53" s="23" t="inlineStr">
+      <c r="B53" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  G_BB_Roulement</t>
         </is>
       </c>
     </row>
     <row r="54" ht="14" customHeight="1">
-      <c r="B54" s="23" t="inlineStr">
+      <c r="B54" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  G_Travaux_Base</t>
         </is>
       </c>
     </row>
     <row r="55" ht="14" customHeight="1">
-      <c r="B55" s="23" t="inlineStr">
+      <c r="B55" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  G_Fond_Forme</t>
         </is>
       </c>
     </row>
     <row r="56" ht="14" customHeight="1">
-      <c r="B56" s="23" t="inlineStr">
+      <c r="B56" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  G_Bordure_Finie</t>
         </is>
       </c>
     </row>
     <row r="57" ht="14" customHeight="1">
-      <c r="B57" s="23" t="inlineStr">
+      <c r="B57" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  G_Bord_Stationnement</t>
         </is>
       </c>
     </row>
     <row r="58" ht="14" customHeight="1">
-      <c r="B58" s="23" t="inlineStr">
+      <c r="B58" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  G_Trottoir_Fini</t>
         </is>
       </c>
     </row>
     <row r="59" ht="14" customHeight="1">
-      <c r="B59" s="23" t="inlineStr">
+      <c r="B59" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  G_Tablier_Fini_60x60</t>
         </is>
       </c>
     </row>
     <row r="60" ht="14" customHeight="1">
-      <c r="B60" s="23" t="inlineStr">
+      <c r="B60" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  G_Radier_Interieur</t>
         </is>
       </c>
     </row>
     <row r="61" ht="14" customHeight="1">
-      <c r="B61" s="23" t="inlineStr">
+      <c r="B61" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  G_Beton_Proprete</t>
         </is>
       </c>
     </row>
     <row r="62" ht="14" customHeight="1">
-      <c r="B62" s="23" t="inlineStr">
+      <c r="B62" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  G_Fond_Fouille</t>
         </is>
       </c>
     </row>
     <row r="63" ht="14" customHeight="1">
-      <c r="B63" s="23" t="inlineStr">
+      <c r="B63" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  G_Bord_Propriete</t>
         </is>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1">
-      <c r="B64" s="24" t="inlineStr">
+      <c r="B64" s="39" t="inlineStr">
         <is>
           <t>COLONNES COTE_DROIT</t>
         </is>
       </c>
     </row>
     <row r="65" ht="14" customHeight="1">
-      <c r="B65" s="25" t="inlineStr">
+      <c r="B65" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  PK</t>
         </is>
       </c>
     </row>
     <row r="66" ht="14" customHeight="1">
-      <c r="B66" s="25" t="inlineStr">
+      <c r="B66" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  AXE_BB</t>
         </is>
       </c>
     </row>
     <row r="67" ht="14" customHeight="1">
-      <c r="B67" s="25" t="inlineStr">
+      <c r="B67" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  AXE_Travaux</t>
         </is>
       </c>
     </row>
     <row r="68" ht="14" customHeight="1">
-      <c r="B68" s="25" t="inlineStr">
+      <c r="B68" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  AXE_Fond_Forme</t>
         </is>
       </c>
     </row>
     <row r="69" ht="14" customHeight="1">
-      <c r="B69" s="25" t="inlineStr">
+      <c r="B69" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  D_BB_Roulement</t>
         </is>
       </c>
     </row>
     <row r="70" ht="14" customHeight="1">
-      <c r="B70" s="25" t="inlineStr">
+      <c r="B70" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  D_Travaux_Base</t>
         </is>
       </c>
     </row>
     <row r="71" ht="14" customHeight="1">
-      <c r="B71" s="25" t="inlineStr">
+      <c r="B71" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  D_Fond_Forme</t>
         </is>
       </c>
     </row>
     <row r="72" ht="14" customHeight="1">
-      <c r="B72" s="25" t="inlineStr">
+      <c r="B72" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  D_Bordure_Finie</t>
         </is>
       </c>
     </row>
     <row r="73" ht="14" customHeight="1">
-      <c r="B73" s="25" t="inlineStr">
+      <c r="B73" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  D_Trottoir_Fini</t>
         </is>
       </c>
     </row>
     <row r="74" ht="14" customHeight="1">
-      <c r="B74" s="25" t="inlineStr">
+      <c r="B74" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  D_Tablier_Fini_40x40</t>
         </is>
       </c>
     </row>
     <row r="75" ht="14" customHeight="1">
-      <c r="B75" s="25" t="inlineStr">
+      <c r="B75" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  D_Radier_Interieur</t>
         </is>
       </c>
     </row>
     <row r="76" ht="14" customHeight="1">
-      <c r="B76" s="25" t="inlineStr">
+      <c r="B76" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  D_Beton_Proprete</t>
         </is>
       </c>
     </row>
     <row r="77" ht="14" customHeight="1">
-      <c r="B77" s="25" t="inlineStr">
+      <c r="B77" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  D_Fond_Fouille</t>
         </is>
       </c>
     </row>
     <row r="78" ht="14" customHeight="1">
-      <c r="B78" s="25" t="inlineStr">
+      <c r="B78" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">  D_Bord_Propriete</t>
         </is>
@@ -7224,1791 +8403,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F67"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="26" t="inlineStr">
-        <is>
-          <t>COORDONNÉES DE L'AXE — Route Urbaine avec Trottoirs — 1.5 km</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="27" t="inlineStr">
-        <is>
-          <t>Système de référence : Lambert 93 (EPSG:2154)  —  Données à renseigner avec les coordonnées réelles du levé</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="28" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="B3" s="28" t="inlineStr">
-        <is>
-          <t>X (m)</t>
-        </is>
-      </c>
-      <c r="C3" s="28" t="inlineStr">
-        <is>
-          <t>Y (m)</t>
-        </is>
-      </c>
-      <c r="D3" s="28" t="inlineStr">
-        <is>
-          <t>Z axe (m)</t>
-        </is>
-      </c>
-      <c r="E3" s="28" t="inlineStr">
-        <is>
-          <t>Gisement (°)</t>
-        </is>
-      </c>
-      <c r="F3" s="28" t="inlineStr">
-        <is>
-          <t>Dist. cumulée (m)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="15" customHeight="1">
-      <c r="A4" s="29" t="inlineStr">
-        <is>
-          <t>Point kilométrique</t>
-        </is>
-      </c>
-      <c r="B4" s="29" t="inlineStr">
-        <is>
-          <t>Lambert 93 — Est</t>
-        </is>
-      </c>
-      <c r="C4" s="29" t="inlineStr">
-        <is>
-          <t>Lambert 93 — Nord</t>
-        </is>
-      </c>
-      <c r="D4" s="29" t="inlineStr">
-        <is>
-          <t>Cote NGF de l'axe chaussée</t>
-        </is>
-      </c>
-      <c r="E4" s="29" t="inlineStr">
-        <is>
-          <t>Direction route (0°=N, 90°=E)</t>
-        </is>
-      </c>
-      <c r="F4" s="29" t="inlineStr">
-        <is>
-          <t>Distance depuis l'origine</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="30" t="inlineStr">
-        <is>
-          <t>0+000</t>
-        </is>
-      </c>
-      <c r="B5" s="31" t="n">
-        <v>841750</v>
-      </c>
-      <c r="C5" s="31" t="n">
-        <v>6518200</v>
-      </c>
-      <c r="D5" s="32" t="n">
-        <v>98.31999999999999</v>
-      </c>
-      <c r="E5" s="33" t="n">
-        <v>355</v>
-      </c>
-      <c r="F5" s="34" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="35" t="inlineStr">
-        <is>
-          <t>0+025</t>
-        </is>
-      </c>
-      <c r="B6" s="36" t="n">
-        <v>841747.862</v>
-      </c>
-      <c r="C6" s="36" t="n">
-        <v>6518224.908</v>
-      </c>
-      <c r="D6" s="37" t="n">
-        <v>98.3</v>
-      </c>
-      <c r="E6" s="38" t="n">
-        <v>355.0937</v>
-      </c>
-      <c r="F6" s="39" t="n">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="35" t="inlineStr">
-        <is>
-          <t>0+050</t>
-        </is>
-      </c>
-      <c r="B7" s="36" t="n">
-        <v>841745.8050000001</v>
-      </c>
-      <c r="C7" s="36" t="n">
-        <v>6518249.824</v>
-      </c>
-      <c r="D7" s="37" t="n">
-        <v>98.28</v>
-      </c>
-      <c r="E7" s="38" t="n">
-        <v>355.1874</v>
-      </c>
-      <c r="F7" s="39" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="35" t="inlineStr">
-        <is>
-          <t>0+075</t>
-        </is>
-      </c>
-      <c r="B8" s="36" t="n">
-        <v>841743.83</v>
-      </c>
-      <c r="C8" s="36" t="n">
-        <v>6518274.746</v>
-      </c>
-      <c r="D8" s="37" t="n">
-        <v>98.26000000000001</v>
-      </c>
-      <c r="E8" s="38" t="n">
-        <v>355.2808</v>
-      </c>
-      <c r="F8" s="39" t="n">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="30" t="inlineStr">
-        <is>
-          <t>0+100</t>
-        </is>
-      </c>
-      <c r="B9" s="31" t="n">
-        <v>841741.9350000001</v>
-      </c>
-      <c r="C9" s="31" t="n">
-        <v>6518299.674</v>
-      </c>
-      <c r="D9" s="32" t="n">
-        <v>98.23999999999999</v>
-      </c>
-      <c r="E9" s="33" t="n">
-        <v>355.374</v>
-      </c>
-      <c r="F9" s="34" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="35" t="inlineStr">
-        <is>
-          <t>0+125</t>
-        </is>
-      </c>
-      <c r="B10" s="36" t="n">
-        <v>841740.121</v>
-      </c>
-      <c r="C10" s="36" t="n">
-        <v>6518324.609</v>
-      </c>
-      <c r="D10" s="37" t="n">
-        <v>98.22</v>
-      </c>
-      <c r="E10" s="38" t="n">
-        <v>355.4668</v>
-      </c>
-      <c r="F10" s="39" t="n">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="35" t="inlineStr">
-        <is>
-          <t>0+150</t>
-        </is>
-      </c>
-      <c r="B11" s="36" t="n">
-        <v>841738.3860000001</v>
-      </c>
-      <c r="C11" s="36" t="n">
-        <v>6518349.55</v>
-      </c>
-      <c r="D11" s="37" t="n">
-        <v>98.2</v>
-      </c>
-      <c r="E11" s="38" t="n">
-        <v>355.5592</v>
-      </c>
-      <c r="F11" s="39" t="n">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="35" t="inlineStr">
-        <is>
-          <t>0+175</t>
-        </is>
-      </c>
-      <c r="B12" s="36" t="n">
-        <v>841736.73</v>
-      </c>
-      <c r="C12" s="36" t="n">
-        <v>6518374.496</v>
-      </c>
-      <c r="D12" s="37" t="n">
-        <v>98.18000000000001</v>
-      </c>
-      <c r="E12" s="38" t="n">
-        <v>355.651</v>
-      </c>
-      <c r="F12" s="39" t="n">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="30" t="inlineStr">
-        <is>
-          <t>0+200</t>
-        </is>
-      </c>
-      <c r="B13" s="31" t="n">
-        <v>841735.151</v>
-      </c>
-      <c r="C13" s="31" t="n">
-        <v>6518399.448</v>
-      </c>
-      <c r="D13" s="32" t="n">
-        <v>98.16</v>
-      </c>
-      <c r="E13" s="33" t="n">
-        <v>355.7422</v>
-      </c>
-      <c r="F13" s="34" t="n">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="35" t="inlineStr">
-        <is>
-          <t>0+225</t>
-        </is>
-      </c>
-      <c r="B14" s="36" t="n">
-        <v>841733.649</v>
-      </c>
-      <c r="C14" s="36" t="n">
-        <v>6518424.405</v>
-      </c>
-      <c r="D14" s="37" t="n">
-        <v>98.14</v>
-      </c>
-      <c r="E14" s="38" t="n">
-        <v>355.8327</v>
-      </c>
-      <c r="F14" s="39" t="n">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="35" t="inlineStr">
-        <is>
-          <t>0+250</t>
-        </is>
-      </c>
-      <c r="B15" s="36" t="n">
-        <v>841732.223</v>
-      </c>
-      <c r="C15" s="36" t="n">
-        <v>6518449.367</v>
-      </c>
-      <c r="D15" s="37" t="n">
-        <v>98.12</v>
-      </c>
-      <c r="E15" s="38" t="n">
-        <v>355.9223</v>
-      </c>
-      <c r="F15" s="39" t="n">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="35" t="inlineStr">
-        <is>
-          <t>0+275</t>
-        </is>
-      </c>
-      <c r="B16" s="36" t="n">
-        <v>841730.87</v>
-      </c>
-      <c r="C16" s="36" t="n">
-        <v>6518474.334</v>
-      </c>
-      <c r="D16" s="37" t="n">
-        <v>98.09999999999999</v>
-      </c>
-      <c r="E16" s="38" t="n">
-        <v>356.0111</v>
-      </c>
-      <c r="F16" s="39" t="n">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="30" t="inlineStr">
-        <is>
-          <t>0+300</t>
-        </is>
-      </c>
-      <c r="B17" s="31" t="n">
-        <v>841729.589</v>
-      </c>
-      <c r="C17" s="31" t="n">
-        <v>6518499.305</v>
-      </c>
-      <c r="D17" s="32" t="n">
-        <v>98.08</v>
-      </c>
-      <c r="E17" s="33" t="n">
-        <v>356.0988</v>
-      </c>
-      <c r="F17" s="34" t="n">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="35" t="inlineStr">
-        <is>
-          <t>0+325</t>
-        </is>
-      </c>
-      <c r="B18" s="36" t="n">
-        <v>841728.379</v>
-      </c>
-      <c r="C18" s="36" t="n">
-        <v>6518524.28</v>
-      </c>
-      <c r="D18" s="37" t="n">
-        <v>98.06</v>
-      </c>
-      <c r="E18" s="38" t="n">
-        <v>356.1855</v>
-      </c>
-      <c r="F18" s="39" t="n">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="35" t="inlineStr">
-        <is>
-          <t>0+350</t>
-        </is>
-      </c>
-      <c r="B19" s="36" t="n">
-        <v>841727.237</v>
-      </c>
-      <c r="C19" s="36" t="n">
-        <v>6518549.259</v>
-      </c>
-      <c r="D19" s="37" t="n">
-        <v>98.04000000000001</v>
-      </c>
-      <c r="E19" s="38" t="n">
-        <v>356.271</v>
-      </c>
-      <c r="F19" s="39" t="n">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="35" t="inlineStr">
-        <is>
-          <t>0+375</t>
-        </is>
-      </c>
-      <c r="B20" s="36" t="n">
-        <v>841726.162</v>
-      </c>
-      <c r="C20" s="36" t="n">
-        <v>6518574.242</v>
-      </c>
-      <c r="D20" s="37" t="n">
-        <v>98.02</v>
-      </c>
-      <c r="E20" s="38" t="n">
-        <v>356.3553</v>
-      </c>
-      <c r="F20" s="39" t="n">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="30" t="inlineStr">
-        <is>
-          <t>0+400</t>
-        </is>
-      </c>
-      <c r="B21" s="31" t="n">
-        <v>841725.15</v>
-      </c>
-      <c r="C21" s="31" t="n">
-        <v>6518599.227</v>
-      </c>
-      <c r="D21" s="32" t="n">
-        <v>98</v>
-      </c>
-      <c r="E21" s="33" t="n">
-        <v>356.4383</v>
-      </c>
-      <c r="F21" s="34" t="n">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="35" t="inlineStr">
-        <is>
-          <t>0+425</t>
-        </is>
-      </c>
-      <c r="B22" s="36" t="n">
-        <v>841724.201</v>
-      </c>
-      <c r="C22" s="36" t="n">
-        <v>6518624.216</v>
-      </c>
-      <c r="D22" s="37" t="n">
-        <v>97.98</v>
-      </c>
-      <c r="E22" s="38" t="n">
-        <v>356.5198</v>
-      </c>
-      <c r="F22" s="39" t="n">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="35" t="inlineStr">
-        <is>
-          <t>0+450</t>
-        </is>
-      </c>
-      <c r="B23" s="36" t="n">
-        <v>841723.311</v>
-      </c>
-      <c r="C23" s="36" t="n">
-        <v>6518649.208</v>
-      </c>
-      <c r="D23" s="37" t="n">
-        <v>97.95999999999999</v>
-      </c>
-      <c r="E23" s="38" t="n">
-        <v>356.5999</v>
-      </c>
-      <c r="F23" s="39" t="n">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="35" t="inlineStr">
-        <is>
-          <t>0+475</t>
-        </is>
-      </c>
-      <c r="B24" s="36" t="n">
-        <v>841722.478</v>
-      </c>
-      <c r="C24" s="36" t="n">
-        <v>6518674.202</v>
-      </c>
-      <c r="D24" s="37" t="n">
-        <v>97.94</v>
-      </c>
-      <c r="E24" s="38" t="n">
-        <v>356.6784</v>
-      </c>
-      <c r="F24" s="39" t="n">
-        <v>475</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="30" t="inlineStr">
-        <is>
-          <t>0+500</t>
-        </is>
-      </c>
-      <c r="B25" s="31" t="n">
-        <v>841721.7</v>
-      </c>
-      <c r="C25" s="31" t="n">
-        <v>6518699.198</v>
-      </c>
-      <c r="D25" s="32" t="n">
-        <v>97.92</v>
-      </c>
-      <c r="E25" s="33" t="n">
-        <v>356.7553</v>
-      </c>
-      <c r="F25" s="34" t="n">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="35" t="inlineStr">
-        <is>
-          <t>0+525</t>
-        </is>
-      </c>
-      <c r="B26" s="36" t="n">
-        <v>841720.972</v>
-      </c>
-      <c r="C26" s="36" t="n">
-        <v>6518724.197</v>
-      </c>
-      <c r="D26" s="37" t="n">
-        <v>97.90000000000001</v>
-      </c>
-      <c r="E26" s="38" t="n">
-        <v>356.8305</v>
-      </c>
-      <c r="F26" s="39" t="n">
-        <v>525</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="35" t="inlineStr">
-        <is>
-          <t>0+550</t>
-        </is>
-      </c>
-      <c r="B27" s="36" t="n">
-        <v>841720.2929999999</v>
-      </c>
-      <c r="C27" s="36" t="n">
-        <v>6518749.197</v>
-      </c>
-      <c r="D27" s="37" t="n">
-        <v>97.88</v>
-      </c>
-      <c r="E27" s="38" t="n">
-        <v>356.9038</v>
-      </c>
-      <c r="F27" s="39" t="n">
-        <v>550</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="35" t="inlineStr">
-        <is>
-          <t>0+575</t>
-        </is>
-      </c>
-      <c r="B28" s="36" t="n">
-        <v>841719.66</v>
-      </c>
-      <c r="C28" s="36" t="n">
-        <v>6518774.199</v>
-      </c>
-      <c r="D28" s="37" t="n">
-        <v>97.86</v>
-      </c>
-      <c r="E28" s="38" t="n">
-        <v>356.9753</v>
-      </c>
-      <c r="F28" s="39" t="n">
-        <v>575</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="30" t="inlineStr">
-        <is>
-          <t>0+600</t>
-        </is>
-      </c>
-      <c r="B29" s="31" t="n">
-        <v>841719.068</v>
-      </c>
-      <c r="C29" s="31" t="n">
-        <v>6518799.202</v>
-      </c>
-      <c r="D29" s="32" t="n">
-        <v>97.84</v>
-      </c>
-      <c r="E29" s="33" t="n">
-        <v>357.0449</v>
-      </c>
-      <c r="F29" s="34" t="n">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="35" t="inlineStr">
-        <is>
-          <t>0+625</t>
-        </is>
-      </c>
-      <c r="B30" s="36" t="n">
-        <v>841718.5159999999</v>
-      </c>
-      <c r="C30" s="36" t="n">
-        <v>6518824.206</v>
-      </c>
-      <c r="D30" s="37" t="n">
-        <v>97.81999999999999</v>
-      </c>
-      <c r="E30" s="38" t="n">
-        <v>357.1125</v>
-      </c>
-      <c r="F30" s="39" t="n">
-        <v>625</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="35" t="inlineStr">
-        <is>
-          <t>0+650</t>
-        </is>
-      </c>
-      <c r="B31" s="36" t="n">
-        <v>841717.999</v>
-      </c>
-      <c r="C31" s="36" t="n">
-        <v>6518849.212</v>
-      </c>
-      <c r="D31" s="37" t="n">
-        <v>97.8</v>
-      </c>
-      <c r="E31" s="38" t="n">
-        <v>357.178</v>
-      </c>
-      <c r="F31" s="39" t="n">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="35" t="inlineStr">
-        <is>
-          <t>0+675</t>
-        </is>
-      </c>
-      <c r="B32" s="36" t="n">
-        <v>841717.514</v>
-      </c>
-      <c r="C32" s="36" t="n">
-        <v>6518874.218</v>
-      </c>
-      <c r="D32" s="37" t="n">
-        <v>97.78</v>
-      </c>
-      <c r="E32" s="38" t="n">
-        <v>357.2414</v>
-      </c>
-      <c r="F32" s="39" t="n">
-        <v>675</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="30" t="inlineStr">
-        <is>
-          <t>0+700</t>
-        </is>
-      </c>
-      <c r="B33" s="31" t="n">
-        <v>841717.058</v>
-      </c>
-      <c r="C33" s="31" t="n">
-        <v>6518899.224</v>
-      </c>
-      <c r="D33" s="32" t="n">
-        <v>97.76000000000001</v>
-      </c>
-      <c r="E33" s="33" t="n">
-        <v>357.3026</v>
-      </c>
-      <c r="F33" s="34" t="n">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="35" t="inlineStr">
-        <is>
-          <t>0+725</t>
-        </is>
-      </c>
-      <c r="B34" s="36" t="n">
-        <v>841716.626</v>
-      </c>
-      <c r="C34" s="36" t="n">
-        <v>6518924.231</v>
-      </c>
-      <c r="D34" s="37" t="n">
-        <v>97.73999999999999</v>
-      </c>
-      <c r="E34" s="38" t="n">
-        <v>357.3616</v>
-      </c>
-      <c r="F34" s="39" t="n">
-        <v>725</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="35" t="inlineStr">
-        <is>
-          <t>0+750</t>
-        </is>
-      </c>
-      <c r="B35" s="36" t="n">
-        <v>841716.216</v>
-      </c>
-      <c r="C35" s="36" t="n">
-        <v>6518949.239</v>
-      </c>
-      <c r="D35" s="37" t="n">
-        <v>97.72</v>
-      </c>
-      <c r="E35" s="38" t="n">
-        <v>357.4182</v>
-      </c>
-      <c r="F35" s="39" t="n">
-        <v>750</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="35" t="inlineStr">
-        <is>
-          <t>0+775</t>
-        </is>
-      </c>
-      <c r="B36" s="36" t="n">
-        <v>841715.824</v>
-      </c>
-      <c r="C36" s="36" t="n">
-        <v>6518974.246</v>
-      </c>
-      <c r="D36" s="37" t="n">
-        <v>97.7</v>
-      </c>
-      <c r="E36" s="38" t="n">
-        <v>357.4725</v>
-      </c>
-      <c r="F36" s="39" t="n">
-        <v>775</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="30" t="inlineStr">
-        <is>
-          <t>0+800</t>
-        </is>
-      </c>
-      <c r="B37" s="31" t="n">
-        <v>841715.4449999999</v>
-      </c>
-      <c r="C37" s="31" t="n">
-        <v>6518999.253</v>
-      </c>
-      <c r="D37" s="32" t="n">
-        <v>97.68000000000001</v>
-      </c>
-      <c r="E37" s="33" t="n">
-        <v>357.5244</v>
-      </c>
-      <c r="F37" s="34" t="n">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="35" t="inlineStr">
-        <is>
-          <t>0+825</t>
-        </is>
-      </c>
-      <c r="B38" s="36" t="n">
-        <v>841715.076</v>
-      </c>
-      <c r="C38" s="36" t="n">
-        <v>6519024.26</v>
-      </c>
-      <c r="D38" s="37" t="n">
-        <v>97.66</v>
-      </c>
-      <c r="E38" s="38" t="n">
-        <v>357.5738</v>
-      </c>
-      <c r="F38" s="39" t="n">
-        <v>825</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="35" t="inlineStr">
-        <is>
-          <t>0+850</t>
-        </is>
-      </c>
-      <c r="B39" s="36" t="n">
-        <v>841714.713</v>
-      </c>
-      <c r="C39" s="36" t="n">
-        <v>6519049.267</v>
-      </c>
-      <c r="D39" s="37" t="n">
-        <v>97.64</v>
-      </c>
-      <c r="E39" s="38" t="n">
-        <v>357.6207</v>
-      </c>
-      <c r="F39" s="39" t="n">
-        <v>850</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="35" t="inlineStr">
-        <is>
-          <t>0+875</t>
-        </is>
-      </c>
-      <c r="B40" s="36" t="n">
-        <v>841714.352</v>
-      </c>
-      <c r="C40" s="36" t="n">
-        <v>6519074.274</v>
-      </c>
-      <c r="D40" s="37" t="n">
-        <v>97.62</v>
-      </c>
-      <c r="E40" s="38" t="n">
-        <v>357.6651</v>
-      </c>
-      <c r="F40" s="39" t="n">
-        <v>875</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="30" t="inlineStr">
-        <is>
-          <t>0+900</t>
-        </is>
-      </c>
-      <c r="B41" s="31" t="n">
-        <v>841713.988</v>
-      </c>
-      <c r="C41" s="31" t="n">
-        <v>6519099.279</v>
-      </c>
-      <c r="D41" s="32" t="n">
-        <v>97.59999999999999</v>
-      </c>
-      <c r="E41" s="33" t="n">
-        <v>357.7068</v>
-      </c>
-      <c r="F41" s="34" t="n">
-        <v>900</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="35" t="inlineStr">
-        <is>
-          <t>0+925</t>
-        </is>
-      </c>
-      <c r="B42" s="36" t="n">
-        <v>841713.618</v>
-      </c>
-      <c r="C42" s="36" t="n">
-        <v>6519124.284</v>
-      </c>
-      <c r="D42" s="37" t="n">
-        <v>97.58</v>
-      </c>
-      <c r="E42" s="38" t="n">
-        <v>357.7459</v>
-      </c>
-      <c r="F42" s="39" t="n">
-        <v>925</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="35" t="inlineStr">
-        <is>
-          <t>0+950</t>
-        </is>
-      </c>
-      <c r="B43" s="36" t="n">
-        <v>841713.2389999999</v>
-      </c>
-      <c r="C43" s="36" t="n">
-        <v>6519149.288</v>
-      </c>
-      <c r="D43" s="37" t="n">
-        <v>97.56</v>
-      </c>
-      <c r="E43" s="38" t="n">
-        <v>357.7823</v>
-      </c>
-      <c r="F43" s="39" t="n">
-        <v>950</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="35" t="inlineStr">
-        <is>
-          <t>0+975</t>
-        </is>
-      </c>
-      <c r="B44" s="36" t="n">
-        <v>841712.844</v>
-      </c>
-      <c r="C44" s="36" t="n">
-        <v>6519174.292</v>
-      </c>
-      <c r="D44" s="37" t="n">
-        <v>97.54000000000001</v>
-      </c>
-      <c r="E44" s="38" t="n">
-        <v>357.816</v>
-      </c>
-      <c r="F44" s="39" t="n">
-        <v>975</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="30" t="inlineStr">
-        <is>
-          <t>1+000</t>
-        </is>
-      </c>
-      <c r="B45" s="31" t="n">
-        <v>841712.431</v>
-      </c>
-      <c r="C45" s="31" t="n">
-        <v>6519199.294</v>
-      </c>
-      <c r="D45" s="32" t="n">
-        <v>97.52</v>
-      </c>
-      <c r="E45" s="33" t="n">
-        <v>357.847</v>
-      </c>
-      <c r="F45" s="34" t="n">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="35" t="inlineStr">
-        <is>
-          <t>1+025</t>
-        </is>
-      </c>
-      <c r="B46" s="36" t="n">
-        <v>841711.995</v>
-      </c>
-      <c r="C46" s="36" t="n">
-        <v>6519224.295</v>
-      </c>
-      <c r="D46" s="37" t="n">
-        <v>97.5</v>
-      </c>
-      <c r="E46" s="38" t="n">
-        <v>357.8751</v>
-      </c>
-      <c r="F46" s="39" t="n">
-        <v>1025</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="35" t="inlineStr">
-        <is>
-          <t>1+050</t>
-        </is>
-      </c>
-      <c r="B47" s="36" t="n">
-        <v>841711.5330000001</v>
-      </c>
-      <c r="C47" s="36" t="n">
-        <v>6519249.295</v>
-      </c>
-      <c r="D47" s="37" t="n">
-        <v>97.48</v>
-      </c>
-      <c r="E47" s="38" t="n">
-        <v>357.9005</v>
-      </c>
-      <c r="F47" s="39" t="n">
-        <v>1050</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="35" t="inlineStr">
-        <is>
-          <t>1+075</t>
-        </is>
-      </c>
-      <c r="B48" s="36" t="n">
-        <v>841711.039</v>
-      </c>
-      <c r="C48" s="36" t="n">
-        <v>6519274.294</v>
-      </c>
-      <c r="D48" s="37" t="n">
-        <v>97.45999999999999</v>
-      </c>
-      <c r="E48" s="38" t="n">
-        <v>357.923</v>
-      </c>
-      <c r="F48" s="39" t="n">
-        <v>1075</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="30" t="inlineStr">
-        <is>
-          <t>1+100</t>
-        </is>
-      </c>
-      <c r="B49" s="31" t="n">
-        <v>841710.5110000001</v>
-      </c>
-      <c r="C49" s="31" t="n">
-        <v>6519299.291</v>
-      </c>
-      <c r="D49" s="32" t="n">
-        <v>97.44</v>
-      </c>
-      <c r="E49" s="33" t="n">
-        <v>357.9427</v>
-      </c>
-      <c r="F49" s="34" t="n">
-        <v>1100</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="35" t="inlineStr">
-        <is>
-          <t>1+125</t>
-        </is>
-      </c>
-      <c r="B50" s="36" t="n">
-        <v>841709.943</v>
-      </c>
-      <c r="C50" s="36" t="n">
-        <v>6519324.287</v>
-      </c>
-      <c r="D50" s="37" t="n">
-        <v>97.42</v>
-      </c>
-      <c r="E50" s="38" t="n">
-        <v>357.9595</v>
-      </c>
-      <c r="F50" s="39" t="n">
-        <v>1125</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="35" t="inlineStr">
-        <is>
-          <t>1+150</t>
-        </is>
-      </c>
-      <c r="B51" s="36" t="n">
-        <v>841709.3320000001</v>
-      </c>
-      <c r="C51" s="36" t="n">
-        <v>6519349.281</v>
-      </c>
-      <c r="D51" s="37" t="n">
-        <v>97.40000000000001</v>
-      </c>
-      <c r="E51" s="38" t="n">
-        <v>357.9734</v>
-      </c>
-      <c r="F51" s="39" t="n">
-        <v>1150</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="35" t="inlineStr">
-        <is>
-          <t>1+175</t>
-        </is>
-      </c>
-      <c r="B52" s="36" t="n">
-        <v>841708.673</v>
-      </c>
-      <c r="C52" s="36" t="n">
-        <v>6519374.273</v>
-      </c>
-      <c r="D52" s="37" t="n">
-        <v>97.38</v>
-      </c>
-      <c r="E52" s="38" t="n">
-        <v>357.9844</v>
-      </c>
-      <c r="F52" s="39" t="n">
-        <v>1175</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="30" t="inlineStr">
-        <is>
-          <t>1+200</t>
-        </is>
-      </c>
-      <c r="B53" s="31" t="n">
-        <v>841707.963</v>
-      </c>
-      <c r="C53" s="31" t="n">
-        <v>6519399.263</v>
-      </c>
-      <c r="D53" s="32" t="n">
-        <v>97.36</v>
-      </c>
-      <c r="E53" s="33" t="n">
-        <v>357.9925</v>
-      </c>
-      <c r="F53" s="34" t="n">
-        <v>1200</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="35" t="inlineStr">
-        <is>
-          <t>1+225</t>
-        </is>
-      </c>
-      <c r="B54" s="36" t="n">
-        <v>841707.198</v>
-      </c>
-      <c r="C54" s="36" t="n">
-        <v>6519424.252</v>
-      </c>
-      <c r="D54" s="37" t="n">
-        <v>97.34</v>
-      </c>
-      <c r="E54" s="38" t="n">
-        <v>357.9977</v>
-      </c>
-      <c r="F54" s="39" t="n">
-        <v>1225</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="35" t="inlineStr">
-        <is>
-          <t>1+250</t>
-        </is>
-      </c>
-      <c r="B55" s="36" t="n">
-        <v>841706.373</v>
-      </c>
-      <c r="C55" s="36" t="n">
-        <v>6519449.238</v>
-      </c>
-      <c r="D55" s="37" t="n">
-        <v>97.31999999999999</v>
-      </c>
-      <c r="E55" s="38" t="n">
-        <v>357.9999</v>
-      </c>
-      <c r="F55" s="39" t="n">
-        <v>1250</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="35" t="inlineStr">
-        <is>
-          <t>1+275</t>
-        </is>
-      </c>
-      <c r="B56" s="36" t="n">
-        <v>841705.486</v>
-      </c>
-      <c r="C56" s="36" t="n">
-        <v>6519474.223</v>
-      </c>
-      <c r="D56" s="37" t="n">
-        <v>97.3</v>
-      </c>
-      <c r="E56" s="38" t="n">
-        <v>357.9992</v>
-      </c>
-      <c r="F56" s="39" t="n">
-        <v>1275</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="30" t="inlineStr">
-        <is>
-          <t>1+300</t>
-        </is>
-      </c>
-      <c r="B57" s="31" t="n">
-        <v>841704.531</v>
-      </c>
-      <c r="C57" s="31" t="n">
-        <v>6519499.205</v>
-      </c>
-      <c r="D57" s="32" t="n">
-        <v>97.28</v>
-      </c>
-      <c r="E57" s="33" t="n">
-        <v>357.9956</v>
-      </c>
-      <c r="F57" s="34" t="n">
-        <v>1300</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="35" t="inlineStr">
-        <is>
-          <t>1+325</t>
-        </is>
-      </c>
-      <c r="B58" s="36" t="n">
-        <v>841703.505</v>
-      </c>
-      <c r="C58" s="36" t="n">
-        <v>6519524.184</v>
-      </c>
-      <c r="D58" s="37" t="n">
-        <v>97.26000000000001</v>
-      </c>
-      <c r="E58" s="38" t="n">
-        <v>357.9891</v>
-      </c>
-      <c r="F58" s="39" t="n">
-        <v>1325</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="35" t="inlineStr">
-        <is>
-          <t>1+350</t>
-        </is>
-      </c>
-      <c r="B59" s="36" t="n">
-        <v>841702.405</v>
-      </c>
-      <c r="C59" s="36" t="n">
-        <v>6519549.161</v>
-      </c>
-      <c r="D59" s="37" t="n">
-        <v>97.23999999999999</v>
-      </c>
-      <c r="E59" s="38" t="n">
-        <v>357.9796</v>
-      </c>
-      <c r="F59" s="39" t="n">
-        <v>1350</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="35" t="inlineStr">
-        <is>
-          <t>1+375</t>
-        </is>
-      </c>
-      <c r="B60" s="36" t="n">
-        <v>841701.227</v>
-      </c>
-      <c r="C60" s="36" t="n">
-        <v>6519574.135</v>
-      </c>
-      <c r="D60" s="37" t="n">
-        <v>97.22</v>
-      </c>
-      <c r="E60" s="38" t="n">
-        <v>357.9672</v>
-      </c>
-      <c r="F60" s="39" t="n">
-        <v>1375</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="30" t="inlineStr">
-        <is>
-          <t>1+400</t>
-        </is>
-      </c>
-      <c r="B61" s="31" t="n">
-        <v>841699.968</v>
-      </c>
-      <c r="C61" s="31" t="n">
-        <v>6519599.106</v>
-      </c>
-      <c r="D61" s="32" t="n">
-        <v>97.2</v>
-      </c>
-      <c r="E61" s="33" t="n">
-        <v>357.952</v>
-      </c>
-      <c r="F61" s="34" t="n">
-        <v>1400</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="35" t="inlineStr">
-        <is>
-          <t>1+425</t>
-        </is>
-      </c>
-      <c r="B62" s="36" t="n">
-        <v>841698.623</v>
-      </c>
-      <c r="C62" s="36" t="n">
-        <v>6519624.074</v>
-      </c>
-      <c r="D62" s="37" t="n">
-        <v>97.18000000000001</v>
-      </c>
-      <c r="E62" s="38" t="n">
-        <v>357.9338</v>
-      </c>
-      <c r="F62" s="39" t="n">
-        <v>1425</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="35" t="inlineStr">
-        <is>
-          <t>1+450</t>
-        </is>
-      </c>
-      <c r="B63" s="36" t="n">
-        <v>841697.1899999999</v>
-      </c>
-      <c r="C63" s="36" t="n">
-        <v>6519649.038</v>
-      </c>
-      <c r="D63" s="37" t="n">
-        <v>97.16</v>
-      </c>
-      <c r="E63" s="38" t="n">
-        <v>357.9128</v>
-      </c>
-      <c r="F63" s="39" t="n">
-        <v>1450</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="35" t="inlineStr">
-        <is>
-          <t>1+475</t>
-        </is>
-      </c>
-      <c r="B64" s="36" t="n">
-        <v>841695.666</v>
-      </c>
-      <c r="C64" s="36" t="n">
-        <v>6519673.999</v>
-      </c>
-      <c r="D64" s="37" t="n">
-        <v>97.14</v>
-      </c>
-      <c r="E64" s="38" t="n">
-        <v>357.8889</v>
-      </c>
-      <c r="F64" s="39" t="n">
-        <v>1475</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="30" t="inlineStr">
-        <is>
-          <t>1+500</t>
-        </is>
-      </c>
-      <c r="B65" s="31" t="n">
-        <v>841694.047</v>
-      </c>
-      <c r="C65" s="31" t="n">
-        <v>6519698.956</v>
-      </c>
-      <c r="D65" s="32" t="n">
-        <v>97.12</v>
-      </c>
-      <c r="E65" s="33" t="n">
-        <v>357.8623</v>
-      </c>
-      <c r="F65" s="34" t="n">
-        <v>1500</v>
-      </c>
-    </row>
-    <row r="67" ht="30" customHeight="1">
-      <c r="A67" s="40" t="inlineStr">
-        <is>
-          <t>IMPORTANT : Ces coordonnées sont générées automatiquement (projet démo). Remplacer par les coordonnées réelles issues du levé topographique ou du GPS.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A3:F65"/>
-  <mergeCells count="3">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A67:F67"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="41" t="inlineStr">
-        <is>
-          <t>DISTANCES TRANSVERSALES / AXE — Route Urbaine avec Trottoirs — 1.5 km</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="14" customHeight="1">
-      <c r="A2" s="42" t="inlineStr">
-        <is>
-          <t>SECTION EN TRAVERS TYPE — Vue schématique (de gauche à droite)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="14" customHeight="1">
-      <c r="A3" s="43" t="inlineStr"/>
-    </row>
-    <row r="4" ht="14" customHeight="1">
-      <c r="A4" s="43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ← GAUCHE (distances négatives)        AXE        DROITE (distances positives) →</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="14" customHeight="1">
-      <c r="A5" s="43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ─────────────────────────────────────── 0 ────────────────────────────────────────</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="14" customHeight="1">
-      <c r="A6" s="43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Bord_Prop_G ... Canal_G ... Bord_Chaussee_G   |   Bord_Chaussee_D ... Canal_D ... Bord_Prop_D</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="44" t="inlineStr">
-        <is>
-          <t>Élément</t>
-        </is>
-      </c>
-      <c r="B7" s="44" t="inlineStr">
-        <is>
-          <t>Distance / axe (m)</t>
-        </is>
-      </c>
-      <c r="C7" s="44" t="inlineStr">
-        <is>
-          <t>Côté</t>
-        </is>
-      </c>
-      <c r="D7" s="44" t="inlineStr">
-        <is>
-          <t>Colonne cote référence</t>
-        </is>
-      </c>
-      <c r="E7" s="44" t="inlineStr">
-        <is>
-          <t>Onglet source</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="45" t="inlineStr">
-        <is>
-          <t>AXE</t>
-        </is>
-      </c>
-      <c r="B8" s="46" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" s="47" t="inlineStr">
-        <is>
-          <t>Axe</t>
-        </is>
-      </c>
-      <c r="D8" s="47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E8" s="47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="48" t="inlineStr">
-        <is>
-          <t>Bord_Chaussee_G</t>
-        </is>
-      </c>
-      <c r="B9" s="49" t="n">
-        <v>-4</v>
-      </c>
-      <c r="C9" s="48" t="inlineStr">
-        <is>
-          <t>Gauche</t>
-        </is>
-      </c>
-      <c r="D9" s="48" t="inlineStr">
-        <is>
-          <t>Tablier_Fini_G</t>
-        </is>
-      </c>
-      <c r="E9" s="48" t="inlineStr">
-        <is>
-          <t>Cote_Gauche</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="50" t="inlineStr">
-        <is>
-          <t>Bord_Chaussee_D</t>
-        </is>
-      </c>
-      <c r="B10" s="51" t="n">
-        <v>4</v>
-      </c>
-      <c r="C10" s="50" t="inlineStr">
-        <is>
-          <t>Droit</t>
-        </is>
-      </c>
-      <c r="D10" s="50" t="inlineStr">
-        <is>
-          <t>Tablier_Fini_D</t>
-        </is>
-      </c>
-      <c r="E10" s="50" t="inlineStr">
-        <is>
-          <t>Cote_Droit</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="48" t="inlineStr">
-        <is>
-          <t>Trottoir_G</t>
-        </is>
-      </c>
-      <c r="B11" s="49" t="n">
-        <v>-4.8</v>
-      </c>
-      <c r="C11" s="48" t="inlineStr">
-        <is>
-          <t>Gauche</t>
-        </is>
-      </c>
-      <c r="D11" s="48" t="inlineStr">
-        <is>
-          <t>Bord_Propriete_G</t>
-        </is>
-      </c>
-      <c r="E11" s="48" t="inlineStr">
-        <is>
-          <t>Cote_Gauche</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="50" t="inlineStr">
-        <is>
-          <t>Trottoir_D</t>
-        </is>
-      </c>
-      <c r="B12" s="51" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="C12" s="50" t="inlineStr">
-        <is>
-          <t>Droit</t>
-        </is>
-      </c>
-      <c r="D12" s="50" t="inlineStr">
-        <is>
-          <t>Bord_Propriete_D</t>
-        </is>
-      </c>
-      <c r="E12" s="50" t="inlineStr">
-        <is>
-          <t>Cote_Droit</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="48" t="inlineStr">
-        <is>
-          <t>Canal_G (80x80)</t>
-        </is>
-      </c>
-      <c r="B13" s="49" t="n">
-        <v>-5.2</v>
-      </c>
-      <c r="C13" s="48" t="inlineStr">
-        <is>
-          <t>Gauche</t>
-        </is>
-      </c>
-      <c r="D13" s="48" t="inlineStr">
-        <is>
-          <t>Tablier_Fini_G</t>
-        </is>
-      </c>
-      <c r="E13" s="48" t="inlineStr">
-        <is>
-          <t>Cote_Gauche</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="50" t="inlineStr">
-        <is>
-          <t>Canal_D (40x40)</t>
-        </is>
-      </c>
-      <c r="B14" s="51" t="n">
-        <v>5</v>
-      </c>
-      <c r="C14" s="50" t="inlineStr">
-        <is>
-          <t>Droit</t>
-        </is>
-      </c>
-      <c r="D14" s="50" t="inlineStr">
-        <is>
-          <t>Tablier_Fini_D</t>
-        </is>
-      </c>
-      <c r="E14" s="50" t="inlineStr">
-        <is>
-          <t>Cote_Droit</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="48" t="inlineStr">
-        <is>
-          <t>Bord_Propriete_G</t>
-        </is>
-      </c>
-      <c r="B15" s="49" t="n">
-        <v>-7</v>
-      </c>
-      <c r="C15" s="48" t="inlineStr">
-        <is>
-          <t>Gauche</t>
-        </is>
-      </c>
-      <c r="D15" s="48" t="inlineStr">
-        <is>
-          <t>Bord_Propriete_G</t>
-        </is>
-      </c>
-      <c r="E15" s="48" t="inlineStr">
-        <is>
-          <t>Cote_Gauche</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="50" t="inlineStr">
-        <is>
-          <t>Bord_Propriete_D</t>
-        </is>
-      </c>
-      <c r="B16" s="51" t="n">
-        <v>7</v>
-      </c>
-      <c r="C16" s="50" t="inlineStr">
-        <is>
-          <t>Droit</t>
-        </is>
-      </c>
-      <c r="D16" s="50" t="inlineStr">
-        <is>
-          <t>Bord_Propriete_D</t>
-        </is>
-      </c>
-      <c r="E16" s="50" t="inlineStr">
-        <is>
-          <t>Cote_Droit</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="52" t="inlineStr">
-        <is>
-          <t>UTILISATION :
-• La colonne 'Distance / axe' donne la position transversale de chaque élément (- = gauche, + = droite).
-• Combinée aux coordonnées XY de PK_Coordonnees, elle permet de calculer la position GPS de chaque élément via : X_elem = X_axe + dist × sin(gisement + 90°) / Y_elem = Y_axe + dist × cos(gisement + 90°).</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="18" customHeight="1"/>
-    <row r="20" ht="18" customHeight="1"/>
-  </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A18:E20"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A3:E3"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>